<commit_message>
ingesta: snapshot 2026-07-23 18:42 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-07-23/CORDOBA_JUL26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-07-23/CORDOBA_JUL26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B162B6-0779-461F-A049-1F44C5D560F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0C8D75-01C5-4909-9911-5CDD2953FA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
   <sheets>
     <sheet name="ENERO_2026" sheetId="1" r:id="rId1"/>
@@ -10023,7 +10023,7 @@
                   <c:v>2.4</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-1</c:v>
+                  <c:v>107.60000000000002</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>-1</c:v>
@@ -19982,7 +19982,9 @@
       <c r="Y3" s="25">
         <v>0</v>
       </c>
-      <c r="Z3" s="25"/>
+      <c r="Z3" s="25">
+        <v>7.9</v>
+      </c>
       <c r="AA3" s="25"/>
       <c r="AB3" s="25"/>
       <c r="AC3" s="25"/>
@@ -19994,7 +19996,7 @@
       <c r="AI3" s="34"/>
       <c r="AJ3" s="36">
         <f>SUM(E3:AI3)</f>
-        <v>118.9</v>
+        <v>126.80000000000001</v>
       </c>
       <c r="AK3" s="30">
         <v>27.817857142857147</v>
@@ -20076,7 +20078,9 @@
       <c r="Y4" s="25">
         <v>0</v>
       </c>
-      <c r="Z4" s="25"/>
+      <c r="Z4" s="25">
+        <v>31.8</v>
+      </c>
       <c r="AA4" s="25"/>
       <c r="AB4" s="25"/>
       <c r="AC4" s="25"/>
@@ -20088,7 +20092,7 @@
       <c r="AI4" s="34"/>
       <c r="AJ4" s="36">
         <f t="shared" ref="AJ4:AJ17" si="0">SUM(E4:AI4)</f>
-        <v>97.399999999999991</v>
+        <v>129.19999999999999</v>
       </c>
       <c r="AK4" s="30">
         <v>47.628571428571419</v>
@@ -20170,7 +20174,9 @@
       <c r="Y5" s="25">
         <v>0</v>
       </c>
-      <c r="Z5" s="25"/>
+      <c r="Z5" s="25">
+        <v>33.200000000000003</v>
+      </c>
       <c r="AA5" s="25"/>
       <c r="AB5" s="25"/>
       <c r="AC5" s="25"/>
@@ -20182,7 +20188,7 @@
       <c r="AI5" s="34"/>
       <c r="AJ5" s="36">
         <f t="shared" si="0"/>
-        <v>172.79999999999998</v>
+        <v>206</v>
       </c>
       <c r="AK5" s="30">
         <v>40.986206896551728</v>
@@ -20264,7 +20270,9 @@
       <c r="Y6" s="25">
         <v>2.4</v>
       </c>
-      <c r="Z6" s="25"/>
+      <c r="Z6" s="25">
+        <v>1.2</v>
+      </c>
       <c r="AA6" s="25"/>
       <c r="AB6" s="25"/>
       <c r="AC6" s="25"/>
@@ -20276,7 +20284,7 @@
       <c r="AI6" s="34"/>
       <c r="AJ6" s="36">
         <f t="shared" si="0"/>
-        <v>117.60000000000001</v>
+        <v>118.80000000000001</v>
       </c>
       <c r="AK6" s="30">
         <v>88.719230769230762</v>
@@ -20462,7 +20470,9 @@
       <c r="Y9" s="25">
         <v>0</v>
       </c>
-      <c r="Z9" s="25"/>
+      <c r="Z9" s="25">
+        <v>0</v>
+      </c>
       <c r="AA9" s="25"/>
       <c r="AB9" s="25"/>
       <c r="AC9" s="25"/>
@@ -20632,7 +20642,9 @@
       <c r="Y11" s="25">
         <v>0</v>
       </c>
-      <c r="Z11" s="25"/>
+      <c r="Z11" s="25">
+        <v>3.4</v>
+      </c>
       <c r="AA11" s="25"/>
       <c r="AB11" s="25"/>
       <c r="AC11" s="25"/>
@@ -20644,7 +20656,7 @@
       <c r="AI11" s="34"/>
       <c r="AJ11" s="36">
         <f t="shared" si="0"/>
-        <v>148</v>
+        <v>151.4</v>
       </c>
       <c r="AK11" s="30">
         <v>19.188461538461539</v>
@@ -20724,7 +20736,9 @@
       <c r="Y12" s="25">
         <v>0</v>
       </c>
-      <c r="Z12" s="25"/>
+      <c r="Z12" s="25">
+        <v>1.4</v>
+      </c>
       <c r="AA12" s="25"/>
       <c r="AB12" s="25"/>
       <c r="AC12" s="25"/>
@@ -20736,7 +20750,7 @@
       <c r="AI12" s="34"/>
       <c r="AJ12" s="36">
         <f t="shared" si="0"/>
-        <v>60</v>
+        <v>61.4</v>
       </c>
       <c r="AK12" s="30">
         <v>34.724137931034484</v>
@@ -20818,7 +20832,9 @@
       <c r="Y13" s="25">
         <v>0</v>
       </c>
-      <c r="Z13" s="25"/>
+      <c r="Z13" s="25">
+        <v>24</v>
+      </c>
       <c r="AA13" s="25"/>
       <c r="AB13" s="25"/>
       <c r="AC13" s="25"/>
@@ -20830,7 +20846,7 @@
       <c r="AI13" s="34"/>
       <c r="AJ13" s="36">
         <f t="shared" si="0"/>
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="AK13" s="30"/>
     </row>
@@ -20910,7 +20926,9 @@
       <c r="Y14" s="25">
         <v>0</v>
       </c>
-      <c r="Z14" s="25"/>
+      <c r="Z14" s="25">
+        <v>0</v>
+      </c>
       <c r="AA14" s="25"/>
       <c r="AB14" s="25"/>
       <c r="AC14" s="25"/>
@@ -21004,7 +21022,9 @@
       <c r="Y15" s="25">
         <v>0</v>
       </c>
-      <c r="Z15" s="25"/>
+      <c r="Z15" s="25">
+        <v>4.7</v>
+      </c>
       <c r="AA15" s="25"/>
       <c r="AB15" s="25"/>
       <c r="AC15" s="25"/>
@@ -21016,7 +21036,7 @@
       <c r="AI15" s="34"/>
       <c r="AJ15" s="36">
         <f t="shared" si="0"/>
-        <v>130.30000000000001</v>
+        <v>135</v>
       </c>
       <c r="AK15" s="30">
         <v>60.46</v>
@@ -21210,7 +21230,7 @@
       </c>
       <c r="Z19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>107.60000000000002</v>
       </c>
       <c r="AA19" s="26">
         <f t="shared" si="1"/>

</xml_diff>